<commit_message>
Customisation du rapport html
</commit_message>
<xml_diff>
--- a/reports/geoaudit_report.xlsx
+++ b/reports/geoaudit_report.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,6 +507,33 @@
         <v>60.71</v>
       </c>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>MOYEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>60.71</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>MOYEN</t>
         </is>
@@ -523,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +620,7 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="3">
@@ -626,7 +653,7 @@
         </is>
       </c>
       <c r="G3" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="4">
@@ -659,7 +686,7 @@
         </is>
       </c>
       <c r="G4" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="5">
@@ -692,7 +719,7 @@
         </is>
       </c>
       <c r="G5" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="6">
@@ -725,7 +752,7 @@
         </is>
       </c>
       <c r="G6" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="7">
@@ -758,7 +785,7 @@
         </is>
       </c>
       <c r="G7" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="8">
@@ -791,7 +818,7 @@
         </is>
       </c>
       <c r="G8" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="9">
@@ -824,7 +851,7 @@
         </is>
       </c>
       <c r="G9" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="10">
@@ -857,7 +884,7 @@
         </is>
       </c>
       <c r="G10" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="11">
@@ -890,7 +917,7 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="12">
@@ -923,7 +950,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="13">
@@ -956,7 +983,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="14">
@@ -989,7 +1016,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="15">
@@ -1022,7 +1049,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="16">
@@ -1055,7 +1082,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="17">
@@ -1088,7 +1115,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46215.63143710565</v>
+        <v>46215.76908900739</v>
       </c>
     </row>
     <row r="18">
@@ -1121,7 +1148,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="19">
@@ -1154,7 +1181,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="20">
@@ -1187,7 +1214,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="21">
@@ -1220,7 +1247,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="22">
@@ -1253,7 +1280,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="23">
@@ -1286,7 +1313,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="24">
@@ -1319,7 +1346,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="25">
@@ -1352,7 +1379,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="26">
@@ -1385,7 +1412,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="27">
@@ -1418,7 +1445,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="28">
@@ -1451,7 +1478,7 @@
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="29">
@@ -1484,7 +1511,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="30">
@@ -1517,7 +1544,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="31">
@@ -1550,7 +1577,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="32">
@@ -1583,7 +1610,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
       </c>
     </row>
     <row r="33">
@@ -1616,7 +1643,535 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46215.63143905852</v>
+        <v>46215.76909200804</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>G001</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>GEOMETRY_VALID</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Nombre de géométries invalides</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>G002</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>EMPTY_GEOMETRY</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Nombre de géométries vides</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>G003</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SRID_CHECK</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1517</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Système de coordonnées différent de EPSG:2154</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>G004</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>GEOMETRY_TYPE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1517</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>POINT</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>G005</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ENTITY_COUNT</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1517</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Nombre total d entités</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>G006</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NULL_GEOMETRY</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Entités sans géométrie</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>G007</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DUPLICATE_GEOMETRY</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Géométries identiques détectées</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>G008</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>COLUMN_COUNT</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>15</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Nombre de colonnes attributaires</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>G009</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NULL_ATTRIBUTES</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1517</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Nombre de lignes avec valeurs NULL</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>G010</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>VERTEX_COUNT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1517</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Nombre total de sommets</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>G011</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SPATIAL_EXTENT</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>BOX(2.1655421457014 48.743385629116,2.538242116570473 48.95756799268)</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>G012</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MULTIPART_GEOMETRY</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Nombre de géométries multiparties</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>G013</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ZERO_AREA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Polygones avec surface nulle</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>G014</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ZERO_LENGTH</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Lignes avec longueur nulle</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>G015</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GEOMETRY_COMPLEXITY</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Nombre maximum de sommets dans une géométrie</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="n">
+        <v>46215.7690938201</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>G016</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>EMPTY_EXTENT</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Vérification de l emprise spatiale</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="n">
+        <v>46215.7690938201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout de d'une interface utilisateur en Streamlit
</commit_message>
<xml_diff>
--- a/reports/geoaudit_report.xlsx
+++ b/reports/geoaudit_report.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,27 +488,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>16</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D3" t="n">
         <v>28</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>32.14</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CRITIQUE</t>
+          <t>MOYEN</t>
         </is>
       </c>
     </row>
@@ -696,60 +696,6 @@
         <v>60.71</v>
       </c>
       <c r="G10" t="inlineStr">
-        <is>
-          <t>MOYEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>16</v>
-      </c>
-      <c r="C11" t="n">
-        <v>15</v>
-      </c>
-      <c r="D11" t="n">
-        <v>28</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" t="n">
-        <v>53.57</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>MOYEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>16</v>
-      </c>
-      <c r="C12" t="n">
-        <v>17</v>
-      </c>
-      <c r="D12" t="n">
-        <v>28</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="n">
-        <v>60.71</v>
-      </c>
-      <c r="G12" t="inlineStr">
         <is>
           <t>MOYEN</t>
         </is>
@@ -766,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G177"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -836,7 +782,7 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="3">
@@ -869,7 +815,7 @@
         </is>
       </c>
       <c r="G3" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="4">
@@ -902,7 +848,7 @@
         </is>
       </c>
       <c r="G4" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="5">
@@ -935,7 +881,7 @@
         </is>
       </c>
       <c r="G5" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="6">
@@ -968,7 +914,7 @@
         </is>
       </c>
       <c r="G6" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="7">
@@ -1001,7 +947,7 @@
         </is>
       </c>
       <c r="G7" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="8">
@@ -1034,7 +980,7 @@
         </is>
       </c>
       <c r="G8" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="9">
@@ -1067,7 +1013,7 @@
         </is>
       </c>
       <c r="G9" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="10">
@@ -1100,7 +1046,7 @@
         </is>
       </c>
       <c r="G10" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="11">
@@ -1133,7 +1079,7 @@
         </is>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="12">
@@ -1166,7 +1112,7 @@
         </is>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="13">
@@ -1199,7 +1145,7 @@
         </is>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="14">
@@ -1232,7 +1178,7 @@
         </is>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="15">
@@ -1265,7 +1211,7 @@
         </is>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="16">
@@ -1298,7 +1244,7 @@
         </is>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="17">
@@ -1331,7 +1277,7 @@
         </is>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46216.41148744745</v>
+        <v>46216.61522897824</v>
       </c>
     </row>
     <row r="18">
@@ -1347,7 +1293,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1364,7 +1310,7 @@
         </is>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="19">
@@ -1380,16 +1326,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>21958</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1397,7 +1343,7 @@
         </is>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="20">
@@ -1413,16 +1359,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>493602</v>
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1430,7 +1376,7 @@
         </is>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="21">
@@ -1446,7 +1392,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1455,7 +1401,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>515560</v>
+        <v>286831</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1463,7 +1409,7 @@
         </is>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="22">
@@ -1479,7 +1425,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1488,7 +1434,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>515560</v>
+        <v>286831</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1496,7 +1442,7 @@
         </is>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="23">
@@ -1512,16 +1458,16 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>21958</v>
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1529,7 +1475,7 @@
         </is>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="24">
@@ -1545,7 +1491,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1554,7 +1500,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>83645</v>
+        <v>4184</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1562,7 +1508,7 @@
         </is>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="25">
@@ -1578,7 +1524,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1587,7 +1533,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1595,7 +1541,7 @@
         </is>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="26">
@@ -1611,7 +1557,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1620,7 +1566,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>515560</v>
+        <v>286831</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1628,7 +1574,7 @@
         </is>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="27">
@@ -1644,7 +1590,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1653,7 +1599,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>493602</v>
+        <v>286831</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1661,7 +1607,7 @@
         </is>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="28">
@@ -1677,7 +1623,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1690,11 +1636,11 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>BOX(1.45074 48.12554,3.51862 49.21537)</t>
+          <t>BOX(598620.1277744038 6868436.5837209765,669264.795726517 6904953.574338398)</t>
         </is>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="29">
@@ -1710,7 +1656,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1727,7 +1673,7 @@
         </is>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="30">
@@ -1743,7 +1689,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1760,7 +1706,7 @@
         </is>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="31">
@@ -1776,7 +1722,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1793,7 +1739,7 @@
         </is>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="32">
@@ -1809,7 +1755,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1826,7 +1772,7 @@
         </is>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="33">
@@ -1842,7 +1788,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>base_equipement</t>
+          <t>base_adresse_95</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1859,7 +1805,7 @@
         </is>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46216.41148930043</v>
+        <v>46216.61523071364</v>
       </c>
     </row>
     <row r="34">
@@ -1892,7 +1838,7 @@
         </is>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="35">
@@ -1925,7 +1871,7 @@
         </is>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="36">
@@ -1958,7 +1904,7 @@
         </is>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="37">
@@ -1991,7 +1937,7 @@
         </is>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="38">
@@ -2024,7 +1970,7 @@
         </is>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="39">
@@ -2057,7 +2003,7 @@
         </is>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="40">
@@ -2090,7 +2036,7 @@
         </is>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="41">
@@ -2123,7 +2069,7 @@
         </is>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="42">
@@ -2156,7 +2102,7 @@
         </is>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="43">
@@ -2189,7 +2135,7 @@
         </is>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="44">
@@ -2222,7 +2168,7 @@
         </is>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="45">
@@ -2255,7 +2201,7 @@
         </is>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="46">
@@ -2288,7 +2234,7 @@
         </is>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="47">
@@ -2321,7 +2267,7 @@
         </is>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="48">
@@ -2354,7 +2300,7 @@
         </is>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="49">
@@ -2387,7 +2333,7 @@
         </is>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46216.4116167965</v>
+        <v>46216.61525909854</v>
       </c>
     </row>
     <row r="50">
@@ -2420,7 +2366,7 @@
         </is>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="51">
@@ -2453,7 +2399,7 @@
         </is>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="52">
@@ -2486,7 +2432,7 @@
         </is>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="53">
@@ -2519,7 +2465,7 @@
         </is>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="54">
@@ -2552,7 +2498,7 @@
         </is>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="55">
@@ -2585,7 +2531,7 @@
         </is>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="56">
@@ -2618,7 +2564,7 @@
         </is>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="57">
@@ -2651,7 +2597,7 @@
         </is>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="58">
@@ -2684,7 +2630,7 @@
         </is>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="59">
@@ -2717,7 +2663,7 @@
         </is>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="60">
@@ -2750,7 +2696,7 @@
         </is>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="61">
@@ -2783,7 +2729,7 @@
         </is>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="62">
@@ -2816,7 +2762,7 @@
         </is>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="63">
@@ -2849,7 +2795,7 @@
         </is>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="64">
@@ -2882,7 +2828,7 @@
         </is>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="65">
@@ -2915,7 +2861,7 @@
         </is>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46216.41161839509</v>
+        <v>46216.6152604887</v>
       </c>
     </row>
     <row r="66">
@@ -2948,7 +2894,7 @@
         </is>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="67">
@@ -2981,7 +2927,7 @@
         </is>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="68">
@@ -3014,7 +2960,7 @@
         </is>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="69">
@@ -3047,7 +2993,7 @@
         </is>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="70">
@@ -3080,7 +3026,7 @@
         </is>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="71">
@@ -3113,7 +3059,7 @@
         </is>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="72">
@@ -3146,7 +3092,7 @@
         </is>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="73">
@@ -3179,7 +3125,7 @@
         </is>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="74">
@@ -3212,7 +3158,7 @@
         </is>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="75">
@@ -3245,7 +3191,7 @@
         </is>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="76">
@@ -3278,7 +3224,7 @@
         </is>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="77">
@@ -3311,7 +3257,7 @@
         </is>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="78">
@@ -3344,7 +3290,7 @@
         </is>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="79">
@@ -3377,7 +3323,7 @@
         </is>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="80">
@@ -3410,7 +3356,7 @@
         </is>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="81">
@@ -3443,7 +3389,7 @@
         </is>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46216.41162092915</v>
+        <v>46216.61526172284</v>
       </c>
     </row>
     <row r="82">
@@ -3476,7 +3422,7 @@
         </is>
       </c>
       <c r="G82" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="83">
@@ -3509,7 +3455,7 @@
         </is>
       </c>
       <c r="G83" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="84">
@@ -3542,7 +3488,7 @@
         </is>
       </c>
       <c r="G84" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="85">
@@ -3575,7 +3521,7 @@
         </is>
       </c>
       <c r="G85" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="86">
@@ -3608,7 +3554,7 @@
         </is>
       </c>
       <c r="G86" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="87">
@@ -3641,7 +3587,7 @@
         </is>
       </c>
       <c r="G87" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="88">
@@ -3674,7 +3620,7 @@
         </is>
       </c>
       <c r="G88" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="89">
@@ -3707,7 +3653,7 @@
         </is>
       </c>
       <c r="G89" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="90">
@@ -3740,7 +3686,7 @@
         </is>
       </c>
       <c r="G90" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="91">
@@ -3773,7 +3719,7 @@
         </is>
       </c>
       <c r="G91" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="92">
@@ -3806,7 +3752,7 @@
         </is>
       </c>
       <c r="G92" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="93">
@@ -3839,7 +3785,7 @@
         </is>
       </c>
       <c r="G93" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="94">
@@ -3872,7 +3818,7 @@
         </is>
       </c>
       <c r="G94" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="95">
@@ -3905,7 +3851,7 @@
         </is>
       </c>
       <c r="G95" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="96">
@@ -3938,7 +3884,7 @@
         </is>
       </c>
       <c r="G96" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="97">
@@ -3971,7 +3917,7 @@
         </is>
       </c>
       <c r="G97" s="1" t="n">
-        <v>46216.41162249682</v>
+        <v>46216.61526323869</v>
       </c>
     </row>
     <row r="98">
@@ -4004,7 +3950,7 @@
         </is>
       </c>
       <c r="G98" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="99">
@@ -4037,7 +3983,7 @@
         </is>
       </c>
       <c r="G99" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="100">
@@ -4070,7 +4016,7 @@
         </is>
       </c>
       <c r="G100" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="101">
@@ -4103,7 +4049,7 @@
         </is>
       </c>
       <c r="G101" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="102">
@@ -4136,7 +4082,7 @@
         </is>
       </c>
       <c r="G102" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="103">
@@ -4169,7 +4115,7 @@
         </is>
       </c>
       <c r="G103" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="104">
@@ -4202,7 +4148,7 @@
         </is>
       </c>
       <c r="G104" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="105">
@@ -4235,7 +4181,7 @@
         </is>
       </c>
       <c r="G105" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="106">
@@ -4268,7 +4214,7 @@
         </is>
       </c>
       <c r="G106" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="107">
@@ -4301,7 +4247,7 @@
         </is>
       </c>
       <c r="G107" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="108">
@@ -4334,7 +4280,7 @@
         </is>
       </c>
       <c r="G108" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="109">
@@ -4367,7 +4313,7 @@
         </is>
       </c>
       <c r="G109" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="110">
@@ -4400,7 +4346,7 @@
         </is>
       </c>
       <c r="G110" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="111">
@@ -4433,7 +4379,7 @@
         </is>
       </c>
       <c r="G111" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="112">
@@ -4466,7 +4412,7 @@
         </is>
       </c>
       <c r="G112" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="113">
@@ -4499,7 +4445,7 @@
         </is>
       </c>
       <c r="G113" s="1" t="n">
-        <v>46216.41162407512</v>
+        <v>46216.6152645746</v>
       </c>
     </row>
     <row r="114">
@@ -4532,7 +4478,7 @@
         </is>
       </c>
       <c r="G114" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="115">
@@ -4565,7 +4511,7 @@
         </is>
       </c>
       <c r="G115" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="116">
@@ -4598,7 +4544,7 @@
         </is>
       </c>
       <c r="G116" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="117">
@@ -4631,7 +4577,7 @@
         </is>
       </c>
       <c r="G117" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="118">
@@ -4664,7 +4610,7 @@
         </is>
       </c>
       <c r="G118" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="119">
@@ -4697,7 +4643,7 @@
         </is>
       </c>
       <c r="G119" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="120">
@@ -4730,7 +4676,7 @@
         </is>
       </c>
       <c r="G120" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="121">
@@ -4763,7 +4709,7 @@
         </is>
       </c>
       <c r="G121" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="122">
@@ -4796,7 +4742,7 @@
         </is>
       </c>
       <c r="G122" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="123">
@@ -4829,7 +4775,7 @@
         </is>
       </c>
       <c r="G123" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="124">
@@ -4862,7 +4808,7 @@
         </is>
       </c>
       <c r="G124" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="125">
@@ -4895,7 +4841,7 @@
         </is>
       </c>
       <c r="G125" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="126">
@@ -4928,7 +4874,7 @@
         </is>
       </c>
       <c r="G126" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="127">
@@ -4961,7 +4907,7 @@
         </is>
       </c>
       <c r="G127" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="128">
@@ -4994,7 +4940,7 @@
         </is>
       </c>
       <c r="G128" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="129">
@@ -5027,7 +4973,7 @@
         </is>
       </c>
       <c r="G129" s="1" t="n">
-        <v>46216.41162567645</v>
+        <v>46216.61526605261</v>
       </c>
     </row>
     <row r="130">
@@ -5060,7 +5006,7 @@
         </is>
       </c>
       <c r="G130" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="131">
@@ -5093,7 +5039,7 @@
         </is>
       </c>
       <c r="G131" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="132">
@@ -5126,7 +5072,7 @@
         </is>
       </c>
       <c r="G132" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="133">
@@ -5159,7 +5105,7 @@
         </is>
       </c>
       <c r="G133" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="134">
@@ -5192,7 +5138,7 @@
         </is>
       </c>
       <c r="G134" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="135">
@@ -5225,7 +5171,7 @@
         </is>
       </c>
       <c r="G135" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="136">
@@ -5258,7 +5204,7 @@
         </is>
       </c>
       <c r="G136" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="137">
@@ -5291,7 +5237,7 @@
         </is>
       </c>
       <c r="G137" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="138">
@@ -5324,7 +5270,7 @@
         </is>
       </c>
       <c r="G138" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="139">
@@ -5357,7 +5303,7 @@
         </is>
       </c>
       <c r="G139" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="140">
@@ -5390,7 +5336,7 @@
         </is>
       </c>
       <c r="G140" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="141">
@@ -5423,7 +5369,7 @@
         </is>
       </c>
       <c r="G141" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="142">
@@ -5456,7 +5402,7 @@
         </is>
       </c>
       <c r="G142" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="143">
@@ -5489,7 +5435,7 @@
         </is>
       </c>
       <c r="G143" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="144">
@@ -5522,7 +5468,7 @@
         </is>
       </c>
       <c r="G144" s="1" t="n">
-        <v>46216.41162742284</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
     <row r="145">
@@ -5555,1063 +5501,7 @@
         </is>
       </c>
       <c r="G145" s="1" t="n">
-        <v>46216.41162742284</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>G001</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>GEOMETRY_VALID</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E146" t="n">
-        <v>0</v>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>Nombre de géométries invalides</t>
-        </is>
-      </c>
-      <c r="G146" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>G002</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>EMPTY_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E147" t="n">
-        <v>0</v>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>Nombre de géométries vides</t>
-        </is>
-      </c>
-      <c r="G147" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>G003</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>SRID_CHECK</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E148" t="n">
-        <v>26605</v>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>Système de coordonnées différent de EPSG:2154</t>
-        </is>
-      </c>
-      <c r="G148" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>G004</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>GEOMETRY_TYPE</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E149" t="n">
-        <v>26605</v>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>POINT</t>
-        </is>
-      </c>
-      <c r="G149" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>G005</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>ENTITY_COUNT</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E150" t="n">
-        <v>26605</v>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>Nombre total d entités</t>
-        </is>
-      </c>
-      <c r="G150" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>G006</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>NULL_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E151" t="n">
-        <v>0</v>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>Entités sans géométrie</t>
-        </is>
-      </c>
-      <c r="G151" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>G007</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>DUPLICATE_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E152" t="n">
-        <v>7</v>
-      </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>Géométries identiques détectées</t>
-        </is>
-      </c>
-      <c r="G152" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>G008</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>COLUMN_COUNT</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E153" t="n">
-        <v>13</v>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>Nombre de colonnes attributaires</t>
-        </is>
-      </c>
-      <c r="G153" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>G009</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>NULL_ATTRIBUTES</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E154" t="n">
-        <v>26605</v>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>Nombre de lignes avec valeurs NULL</t>
-        </is>
-      </c>
-      <c r="G154" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>G010</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>VERTEX_COUNT</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E155" t="n">
-        <v>26605</v>
-      </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>Nombre total de sommets</t>
-        </is>
-      </c>
-      <c r="G155" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>G011</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>SPATIAL_EXTENT</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E156" t="n">
-        <v>1</v>
-      </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>BOX(1.541833 48.14828359999995,3.3514197 49.16243079998701)</t>
-        </is>
-      </c>
-      <c r="G156" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>G012</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>MULTIPART_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E157" t="n">
-        <v>0</v>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>Nombre de géométries multiparties</t>
-        </is>
-      </c>
-      <c r="G157" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>G013</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>ZERO_AREA</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E158" t="n">
-        <v>0</v>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>Polygones avec surface nulle</t>
-        </is>
-      </c>
-      <c r="G158" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>G014</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>ZERO_LENGTH</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E159" t="n">
-        <v>0</v>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>Lignes avec longueur nulle</t>
-        </is>
-      </c>
-      <c r="G159" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>G015</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>GEOMETRY_COMPLEXITY</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E160" t="n">
-        <v>1</v>
-      </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>Nombre maximum de sommets dans une géométrie</t>
-        </is>
-      </c>
-      <c r="G160" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>G016</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>EMPTY_EXTENT</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>stationnement_velo_en_ile_de_france</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E161" t="n">
-        <v>0</v>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>Vérification de l emprise spatiale</t>
-        </is>
-      </c>
-      <c r="G161" s="1" t="n">
-        <v>46216.41162945395</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>G001</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>GEOMETRY_VALID</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E162" t="n">
-        <v>0</v>
-      </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>Nombre de géométries invalides</t>
-        </is>
-      </c>
-      <c r="G162" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>G002</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>EMPTY_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E163" t="n">
-        <v>0</v>
-      </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>Nombre de géométries vides</t>
-        </is>
-      </c>
-      <c r="G163" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>G003</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>SRID_CHECK</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E164" t="n">
-        <v>1517</v>
-      </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>Système de coordonnées différent de EPSG:2154</t>
-        </is>
-      </c>
-      <c r="G164" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>G004</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>GEOMETRY_TYPE</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E165" t="n">
-        <v>1517</v>
-      </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>POINT</t>
-        </is>
-      </c>
-      <c r="G165" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>G005</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>ENTITY_COUNT</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E166" t="n">
-        <v>1517</v>
-      </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>Nombre total d entités</t>
-        </is>
-      </c>
-      <c r="G166" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>G006</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>NULL_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E167" t="n">
-        <v>0</v>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>Entités sans géométrie</t>
-        </is>
-      </c>
-      <c r="G167" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>G007</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>DUPLICATE_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E168" t="n">
-        <v>0</v>
-      </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>Géométries identiques détectées</t>
-        </is>
-      </c>
-      <c r="G168" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>G008</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>COLUMN_COUNT</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E169" t="n">
-        <v>15</v>
-      </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>Nombre de colonnes attributaires</t>
-        </is>
-      </c>
-      <c r="G169" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>G009</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>NULL_ATTRIBUTES</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E170" t="n">
-        <v>1517</v>
-      </c>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>Nombre de lignes avec valeurs NULL</t>
-        </is>
-      </c>
-      <c r="G170" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>G010</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>VERTEX_COUNT</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E171" t="n">
-        <v>1517</v>
-      </c>
-      <c r="F171" t="inlineStr">
-        <is>
-          <t>Nombre total de sommets</t>
-        </is>
-      </c>
-      <c r="G171" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>G011</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>SPATIAL_EXTENT</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E172" t="n">
-        <v>1</v>
-      </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>BOX(2.1655421457014 48.743385629116,2.538242116570473 48.95756799268)</t>
-        </is>
-      </c>
-      <c r="G172" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>G012</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>MULTIPART_GEOMETRY</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E173" t="n">
-        <v>0</v>
-      </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>Nombre de géométries multiparties</t>
-        </is>
-      </c>
-      <c r="G173" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>G013</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>ZERO_AREA</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E174" t="n">
-        <v>0</v>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>Polygones avec surface nulle</t>
-        </is>
-      </c>
-      <c r="G174" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>G014</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>ZERO_LENGTH</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E175" t="n">
-        <v>0</v>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>Lignes avec longueur nulle</t>
-        </is>
-      </c>
-      <c r="G175" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>G015</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>GEOMETRY_COMPLEXITY</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="E176" t="n">
-        <v>1</v>
-      </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>Nombre maximum de sommets dans une géométrie</t>
-        </is>
-      </c>
-      <c r="G176" s="1" t="n">
-        <v>46216.41163247747</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>G016</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>EMPTY_EXTENT</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>velib_velos_et_bornes_disponibilite_temps_reel</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E177" t="n">
-        <v>0</v>
-      </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>Vérification de l emprise spatiale</t>
-        </is>
-      </c>
-      <c r="G177" s="1" t="n">
-        <v>46216.41163247747</v>
+        <v>46216.61526755332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>